<commit_message>
Update story content and UI
</commit_message>
<xml_diff>
--- a/md/Timeline.xlsx
+++ b/md/Timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\web\md\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FA30E6C-C048-4FCB-B460-56B16DA038C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49584BFB-2C5B-47F6-857F-12AE91C119FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{D3BAEDBF-A3F9-4F63-9C5F-AA48004A35D0}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="21795" windowHeight="12975" xr2:uid="{D3BAEDBF-A3F9-4F63-9C5F-AA48004A35D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>